<commit_message>
Update TIGPS paper analysis artifacts
</commit_message>
<xml_diff>
--- a/20251229_new_progress/Code/paper_data_newdata/main_paper_results/01_model_performance/02_logistic_decomposed_groups/outputs/logistic_decomposed_groups_performance.xlsx
+++ b/20251229_new_progress/Code/paper_data_newdata/main_paper_results/01_model_performance/02_logistic_decomposed_groups/outputs/logistic_decomposed_groups_performance.xlsx
@@ -670,117 +670,117 @@
         <v>6603</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="I2" s="3" t="inlineStr"/>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>0.816</t>
+          <t>0.831</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
+          <t>0.745</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>0.761</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>0.771</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>0.766</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>0.743</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>0.741</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>0.016</t>
+        </is>
+      </c>
+      <c r="R2" s="3" t="inlineStr">
+        <is>
           <t>0.740</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
-        <is>
-          <t>0.754</t>
-        </is>
-      </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>0.769</t>
-        </is>
-      </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="S2" s="3" t="inlineStr">
+        <is>
+          <t>0.015</t>
+        </is>
+      </c>
+      <c r="T2" s="3" t="inlineStr">
+        <is>
+          <t>0.761</t>
+        </is>
+      </c>
+      <c r="U2" s="3" t="inlineStr">
+        <is>
+          <t>0.017</t>
+        </is>
+      </c>
+      <c r="V2" s="3" t="inlineStr">
+        <is>
+          <t>0.819</t>
+        </is>
+      </c>
+      <c r="W2" s="3" t="inlineStr">
+        <is>
+          <t>0.015</t>
+        </is>
+      </c>
+      <c r="X2" s="3" t="inlineStr">
         <is>
           <t>0.762</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
-        <is>
-          <t>0.737</t>
-        </is>
-      </c>
-      <c r="P2" s="3" t="inlineStr">
-        <is>
-          <t>0.734</t>
-        </is>
-      </c>
-      <c r="Q2" s="3" t="inlineStr">
-        <is>
-          <t>0.018</t>
-        </is>
-      </c>
-      <c r="R2" s="3" t="inlineStr">
-        <is>
-          <t>0.731</t>
-        </is>
-      </c>
-      <c r="S2" s="3" t="inlineStr">
-        <is>
-          <t>0.017</t>
-        </is>
-      </c>
-      <c r="T2" s="3" t="inlineStr">
-        <is>
-          <t>0.755</t>
-        </is>
-      </c>
-      <c r="U2" s="3" t="inlineStr">
-        <is>
-          <t>0.018</t>
-        </is>
-      </c>
-      <c r="V2" s="3" t="inlineStr">
-        <is>
-          <t>0.811</t>
-        </is>
-      </c>
-      <c r="W2" s="3" t="inlineStr">
-        <is>
-          <t>0.015</t>
-        </is>
-      </c>
-      <c r="X2" s="3" t="inlineStr">
-        <is>
-          <t>0.752</t>
-        </is>
-      </c>
       <c r="Y2" s="3" t="inlineStr">
         <is>
-          <t>0.014</t>
+          <t>0.011</t>
         </is>
       </c>
       <c r="Z2" s="3" t="inlineStr">
         <is>
-          <t>0.758</t>
+          <t>0.759</t>
         </is>
       </c>
       <c r="AA2" s="3" t="inlineStr">
         <is>
-          <t>0.023</t>
+          <t>0.027</t>
         </is>
       </c>
       <c r="AB2" s="3" t="inlineStr">
         <is>
-          <t>0.758</t>
+          <t>0.759</t>
         </is>
       </c>
       <c r="AC2" s="3" t="inlineStr">
         <is>
-          <t>0.023</t>
+          <t>0.027</t>
         </is>
       </c>
       <c r="AD2" s="3" t="inlineStr">
         <is>
-          <t>0.705</t>
+          <t>0.720</t>
         </is>
       </c>
       <c r="AE2" s="3" t="inlineStr">
         <is>
-          <t>0.016</t>
+          <t>0.012</t>
         </is>
       </c>
     </row>
@@ -819,7 +819,7 @@
         <v>6603</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="I3" s="3" t="inlineStr"/>
       <c r="J3" s="3" t="inlineStr">
@@ -834,17 +834,17 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>0.669</t>
+          <t>0.670</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>0.682</t>
+          <t>0.679</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>0.676</t>
+          <t>0.675</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr">
@@ -854,82 +854,82 @@
       </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>0.650</t>
+          <t>0.649</t>
         </is>
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>0.013</t>
+          <t>0.016</t>
         </is>
       </c>
       <c r="R3" s="3" t="inlineStr">
         <is>
-          <t>0.649</t>
+          <t>0.648</t>
         </is>
       </c>
       <c r="S3" s="3" t="inlineStr">
         <is>
-          <t>0.013</t>
+          <t>0.016</t>
         </is>
       </c>
       <c r="T3" s="3" t="inlineStr">
         <is>
-          <t>0.669</t>
+          <t>0.668</t>
         </is>
       </c>
       <c r="U3" s="3" t="inlineStr">
         <is>
-          <t>0.013</t>
+          <t>0.017</t>
         </is>
       </c>
       <c r="V3" s="3" t="inlineStr">
         <is>
-          <t>0.707</t>
+          <t>0.710</t>
         </is>
       </c>
       <c r="W3" s="3" t="inlineStr">
         <is>
-          <t>0.011</t>
+          <t>0.012</t>
         </is>
       </c>
       <c r="X3" s="3" t="inlineStr">
         <is>
-          <t>0.666</t>
+          <t>0.664</t>
         </is>
       </c>
       <c r="Y3" s="3" t="inlineStr">
         <is>
-          <t>0.012</t>
+          <t>0.014</t>
         </is>
       </c>
       <c r="Z3" s="3" t="inlineStr">
         <is>
-          <t>0.673</t>
+          <t>0.672</t>
         </is>
       </c>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>0.013</t>
+          <t>0.021</t>
         </is>
       </c>
       <c r="AB3" s="3" t="inlineStr">
         <is>
-          <t>0.673</t>
+          <t>0.672</t>
         </is>
       </c>
       <c r="AC3" s="3" t="inlineStr">
         <is>
-          <t>0.013</t>
+          <t>0.021</t>
         </is>
       </c>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>0.625</t>
+          <t>0.623</t>
         </is>
       </c>
       <c r="AE3" s="3" t="inlineStr">
         <is>
-          <t>0.014</t>
+          <t>0.017</t>
         </is>
       </c>
     </row>
@@ -944,12 +944,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H61"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>0.0292</t>
+          <t>0.0183</t>
         </is>
       </c>
     </row>
@@ -1059,7 +1059,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Instant Response Pressure</t>
+          <t>Distress from Missing Online Events</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>-0.1376</t>
+          <t>-0.1370</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Delinquent and Health-Risk Behaviors</t>
+          <t>Delinquent and Risk Behaviors</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>0.1009</t>
+          <t>0.0789</t>
         </is>
       </c>
     </row>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>0.1472</t>
+          <t>0.1189</t>
         </is>
       </c>
     </row>
@@ -1205,7 +1205,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>-0.2942</t>
+          <t>-0.2618</t>
         </is>
       </c>
     </row>
@@ -1247,7 +1247,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>-0.0933</t>
+          <t>-0.0842</t>
         </is>
       </c>
     </row>
@@ -1269,7 +1269,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Cyberbullying Victimization (including Misinformation-related)</t>
+          <t>Cyberbullying Victimization</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>0.1598</t>
+          <t>0.1183</t>
         </is>
       </c>
     </row>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Cyberbullying Perpetration (including Misinformation-related)</t>
+          <t>Cyberbullying Perpetration</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -1331,7 +1331,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>0.0633</t>
+          <t>0.0702</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1373,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>-0.7664</t>
+          <t>-0.7333</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1415,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>0.3320</t>
+          <t>0.3424</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>0.0265</t>
+          <t>0.0176</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>-0.0394</t>
+          <t>-0.0132</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1541,7 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>-0.0286</t>
+          <t>-0.0305</t>
         </is>
       </c>
     </row>
@@ -1563,7 +1563,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Physical/Offline Bullying Victimization</t>
+          <t>Offline Bullying Victimization</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>0.0985</t>
+          <t>-0.0060</t>
         </is>
       </c>
     </row>
@@ -1625,7 +1625,7 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>-0.0117</t>
+          <t>0.0072</t>
         </is>
       </c>
     </row>
@@ -1667,7 +1667,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>-0.2880</t>
+          <t>-0.3016</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>0.0137</t>
+          <t>0.0091</t>
         </is>
       </c>
     </row>
@@ -1726,32 +1726,32 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>feature_v23_A</t>
+          <t>feature_v9</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Selective Positive Sharing</t>
+          <t>School Belonging and School Identification</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>v23_A</t>
+          <t>v9</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>decomposed_subscale</t>
+          <t>scale_or_single_item</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>v23_1;v23_2;v23_3</t>
+          <t>v9_1;v9_2;v9_3</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>-0.0283</t>
+          <t>-0.0100</t>
         </is>
       </c>
     </row>
@@ -1768,32 +1768,32 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>feature_v23_B</t>
+          <t>feature_v12</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Digital Image Enhancement</t>
+          <t>Classmate Support and Trust</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>v23_B</t>
+          <t>v12</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>decomposed_subscale</t>
+          <t>scale_or_single_item</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>v23_4;v23_5;v23_6</t>
+          <t>v12_1;v12_2;v12_3</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>-0.0398</t>
+          <t>-0.1017</t>
         </is>
       </c>
     </row>
@@ -1810,32 +1810,32 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>feature_v23_C</t>
+          <t>feature_v8_03-v8_06</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Social Feedback Dependency</t>
+          <t>School Social Adversity and Peer Stress Events</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>v23_C</t>
+          <t>v8_03-v8_06</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>decomposed_subscale</t>
+          <t>direct_feature</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>v23_7;v23_8;v23_9</t>
+          <t>v8_03;v8_04;v8_05;v8_06</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>0.0778</t>
+          <t>0.3666</t>
         </is>
       </c>
     </row>
@@ -1852,32 +1852,32 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>feature_v36</t>
+          <t>feature_v23_A</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Physical/Offline Bullying Perpetration</t>
+          <t>Selective Positive Sharing</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>v36</t>
+          <t>v23_A</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>scale_or_single_item</t>
+          <t>decomposed_subscale</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>v36</t>
+          <t>v23_1;v23_2;v23_3</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>0.1051</t>
+          <t>-0.0401</t>
         </is>
       </c>
     </row>
@@ -1894,17 +1894,17 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>feature_v26_A</t>
+          <t>feature_v23_B</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Online Upward Social Comparison</t>
+          <t>Authentic and Less-Ideal Self-Presentation</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>v26_A</t>
+          <t>v23_B</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -1914,12 +1914,12 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>v26_1;v26_2;v26_3</t>
+          <t>v23_4;v23_5;v23_6</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>-0.0541</t>
+          <t>-0.0459</t>
         </is>
       </c>
     </row>
@@ -1936,17 +1936,17 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>feature_v26_B</t>
+          <t>feature_v23_C</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Online Perspective Seeking</t>
+          <t>Covert Social Media Monitoring and Passive Participation</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>v26_B</t>
+          <t>v23_C</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -1956,12 +1956,12 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>v26_4;v26_5;v26_6</t>
+          <t>v23_7;v23_8;v23_9</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>0.2459</t>
+          <t>0.0858</t>
         </is>
       </c>
     </row>
@@ -1978,32 +1978,32 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>feature_v54_A</t>
+          <t>feature_v36</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Self-Awareness</t>
+          <t>Offline Bullying Perpetration</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>v54_A</t>
+          <t>v36</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>decomposed_subscale</t>
+          <t>scale_or_single_item</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>v54_1;v54_2;v54_3;v54_18</t>
+          <t>v36</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>0.6340</t>
+          <t>0.0742</t>
         </is>
       </c>
     </row>
@@ -2020,17 +2020,17 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>feature_v54_B</t>
+          <t>feature_v26_A</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Self-Management</t>
+          <t>Online Upward Social Comparison</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>v54_B</t>
+          <t>v26_A</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -2040,12 +2040,12 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>v54_4;v54_5;v54_6</t>
+          <t>v26_1;v26_2;v26_3</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>-0.3965</t>
+          <t>-0.0685</t>
         </is>
       </c>
     </row>
@@ -2062,17 +2062,17 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>feature_v54_C</t>
+          <t>feature_v26_B</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Motivation &amp; Goal Setting</t>
+          <t>Online Perspective Seeking</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>v54_C</t>
+          <t>v26_B</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -2082,12 +2082,12 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>v54_7;v54_8;v54_9</t>
+          <t>v26_4;v26_5;v26_6</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>0.0272</t>
+          <t>0.2527</t>
         </is>
       </c>
     </row>
@@ -2104,17 +2104,17 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>feature_v54_D</t>
+          <t>feature_v54_A</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Social Awareness &amp; Relationship Skills</t>
+          <t>Self-Awareness</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>v54_D</t>
+          <t>v54_A</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -2124,12 +2124,12 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>v54_10;v54_11;v54_13;v54_14;v54_15</t>
+          <t>v54_1;v54_2;v54_3</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>0.0855</t>
+          <t>0.4988</t>
         </is>
       </c>
     </row>
@@ -2146,17 +2146,17 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>feature_v54_E</t>
+          <t>feature_v54_B</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Help-Seeking</t>
+          <t>Self-Management</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>v54_E</t>
+          <t>v54_B</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -2166,12 +2166,12 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>v54_12;v54_16</t>
+          <t>v54_4;v54_5;v54_6</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>-0.2392</t>
+          <t>-0.3714</t>
         </is>
       </c>
     </row>
@@ -2188,17 +2188,17 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>feature_v54_F</t>
+          <t>feature_v54_C</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Responsible Decision-Making</t>
+          <t>Motivation &amp; Goal Setting</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>v54_F</t>
+          <t>v54_C</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -2208,12 +2208,12 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>v54_17;v54_19;v54_20</t>
+          <t>v54_7;v54_8;v54_9</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>-0.0978</t>
+          <t>-0.0120</t>
         </is>
       </c>
     </row>
@@ -2230,59 +2230,59 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>feature_v22</t>
+          <t>feature_v54_D</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Online Coping and Support Seeking under Distress</t>
+          <t>Social Awareness &amp; Relationship Skills</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>v22</t>
+          <t>v54_D</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>scale_or_single_item</t>
+          <t>decomposed_subscale</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>v22_1;v22_2;v22_3;v22_4;v22_5;v22_6</t>
+          <t>v54_10;v54_11;v54_13;v54_14;v54_15</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>0.1588</t>
+          <t>0.1330</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>W2 -&gt; W3</t>
+          <t>W2 -&gt; W2</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>w2_predict_w3</t>
+          <t>w2_predict_w2</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>feature_v27_A</t>
+          <t>feature_v54_E</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Fear of Missing Out &amp; Social Anxiety</t>
+          <t>Help-Seeking</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>v27_A</t>
+          <t>v54_E</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
@@ -2292,39 +2292,39 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>v27_1;v27_2;v27_3</t>
+          <t>v54_12;v54_16</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>0.0587</t>
+          <t>-0.2653</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>W2 -&gt; W3</t>
+          <t>W2 -&gt; W2</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>w2_predict_w3</t>
+          <t>w2_predict_w2</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>feature_v27_B</t>
+          <t>feature_v54_F</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Instant Response Pressure</t>
+          <t>Responsible Decision-Making</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>v27_B</t>
+          <t>v54_F</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
@@ -2334,39 +2334,39 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>v27_4</t>
+          <t>v54_17;v54_18;v54_19;v54_20</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>-0.0359</t>
+          <t>0.0689</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>W2 -&gt; W3</t>
+          <t>W2 -&gt; W2</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>w2_predict_w3</t>
+          <t>w2_predict_w2</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>feature_v42</t>
+          <t>feature_v22</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Delinquent and Health-Risk Behaviors</t>
+          <t>Online Coping and Emotion Regulation under Distress</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>v42</t>
+          <t>v22</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
@@ -2376,12 +2376,12 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>v42_01;v42_02;v42_03;v42_04;v42_05;v42_06;v42_07;v42_08;v42_09;v42_10;v42_11;v42_12;v42_13</t>
+          <t>v22_1;v22_2;v22_3;v22_4;v22_5;v22_6</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>0.0957</t>
+          <t>0.1419</t>
         </is>
       </c>
     </row>
@@ -2398,32 +2398,32 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>feature_v6</t>
+          <t>feature_v27_A</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Parenting Practices and Parent–Child Interaction Quality (Support/Conflict/Monitoring)</t>
+          <t>Fear of Missing Out &amp; Social Anxiety</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>v6</t>
+          <t>v27_A</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>scale_or_single_item</t>
+          <t>decomposed_subscale</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>v6_1;v6_2;v6_3;v6_4;v6_5;v6_6;v6_7;v6_8;v6_9;v6_10</t>
+          <t>v27_1;v27_2;v27_3</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>0.0653</t>
+          <t>0.0543</t>
         </is>
       </c>
     </row>
@@ -2440,32 +2440,32 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>feature_v5</t>
+          <t>feature_v27_B</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Family Cohesion and Support (Family Functioning)</t>
+          <t>Distress from Missing Online Events</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>v5</t>
+          <t>v27_B</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>scale_or_single_item</t>
+          <t>decomposed_subscale</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>v5_1;v5_2;v5_3;v5_4;v5_5;v5_6</t>
+          <t>v27_4</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>-0.1275</t>
+          <t>-0.0356</t>
         </is>
       </c>
     </row>
@@ -2482,17 +2482,17 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>feature_v49</t>
+          <t>feature_v42</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Perceived Effectiveness of School-based Digital/Technology Learning</t>
+          <t>Delinquent and Risk Behaviors</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>v49</t>
+          <t>v42</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
@@ -2502,12 +2502,12 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>v49</t>
+          <t>v42_01;v42_02;v42_03;v42_04;v42_05;v42_06;v42_07;v42_08;v42_09;v42_10;v42_11;v42_12;v42_13</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>-0.0627</t>
+          <t>0.0860</t>
         </is>
       </c>
     </row>
@@ -2524,17 +2524,17 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>feature_v38</t>
+          <t>feature_v6</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Cyberbullying Victimization (including Misinformation-related)</t>
+          <t>Parenting Practices and Parent–Child Interaction Quality (Support/Conflict/Monitoring)</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>v38</t>
+          <t>v6</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
@@ -2544,12 +2544,12 @@
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>v38</t>
+          <t>v6_1;v6_2;v6_3;v6_4;v6_5;v6_6;v6_7;v6_8;v6_9;v6_10</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>0.0511</t>
+          <t>0.0533</t>
         </is>
       </c>
     </row>
@@ -2566,17 +2566,17 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>feature_v40</t>
+          <t>feature_v5</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Cyberbullying Perpetration (including Misinformation-related)</t>
+          <t>Family Cohesion and Support (Family Functioning)</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>v40</t>
+          <t>v5</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
@@ -2586,12 +2586,12 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>v40</t>
+          <t>v5_1;v5_2;v5_3;v5_4;v5_5;v5_6</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>0.0523</t>
+          <t>-0.1077</t>
         </is>
       </c>
     </row>
@@ -2608,17 +2608,17 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>feature_v52</t>
+          <t>feature_v49</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Self-Worth and Positive Self-Concept</t>
+          <t>Perceived Effectiveness of School-based Digital/Technology Learning</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>v52</t>
+          <t>v49</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
@@ -2628,12 +2628,12 @@
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>v52_1;v52_2;v52_3</t>
+          <t>v49</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>-0.3784</t>
+          <t>-0.0496</t>
         </is>
       </c>
     </row>
@@ -2650,17 +2650,17 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>feature_v28</t>
+          <t>feature_v38</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Problematic Internet Use and Internet Dependence</t>
+          <t>Cyberbullying Victimization</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>v28</t>
+          <t>v38</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
@@ -2670,12 +2670,12 @@
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>v28_1;v28_2;v28_3;v28_4;v28_5;v28_6;v28_7;v28_8;v28_9;v28_10</t>
+          <t>v38</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>0.1316</t>
+          <t>0.0343</t>
         </is>
       </c>
     </row>
@@ -2692,32 +2692,32 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>feature_v25_A</t>
+          <t>feature_v40</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Online Ideal Self-Presentation</t>
+          <t>Cyberbullying Perpetration</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>v25_A</t>
+          <t>v40</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>decomposed_subscale</t>
+          <t>scale_or_single_item</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>v25_1;v25_2;v25_3</t>
+          <t>v40</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>0.0108</t>
+          <t>0.0542</t>
         </is>
       </c>
     </row>
@@ -2734,32 +2734,32 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>feature_v25_B</t>
+          <t>feature_v52</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Real-life Self-Satisfaction</t>
+          <t>Self-Worth and Positive Self-Concept</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>v25_B</t>
+          <t>v52</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>decomposed_subscale</t>
+          <t>scale_or_single_item</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>v25_4;v25_5;v25_6</t>
+          <t>v52_1;v52_2;v52_3</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>-0.1243</t>
+          <t>-0.3572</t>
         </is>
       </c>
     </row>
@@ -2776,32 +2776,32 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>feature_v25_C</t>
+          <t>feature_v28</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Online-Offline Discrepancy &amp; Immersion</t>
+          <t>Problematic Internet Use and Internet Dependence</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>v25_C</t>
+          <t>v28</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>decomposed_subscale</t>
+          <t>scale_or_single_item</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>v25_7;v25_8;v25_9;v25_10;v25_11;v25_12;v25_13;v25_14;v25_15</t>
+          <t>v28_1;v28_2;v28_3;v28_4;v28_5;v28_6;v28_7;v28_8;v28_9;v28_10</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>0.0756</t>
+          <t>0.1346</t>
         </is>
       </c>
     </row>
@@ -2818,32 +2818,32 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>feature_v34</t>
+          <t>feature_v25_A</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Physical/Offline Bullying Victimization</t>
+          <t>Online Ideal Self-Presentation</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>v34</t>
+          <t>v25_A</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>scale_or_single_item</t>
+          <t>decomposed_subscale</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>v34</t>
+          <t>v25_1;v25_2;v25_3</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>0.0628</t>
+          <t>0.0094</t>
         </is>
       </c>
     </row>
@@ -2860,32 +2860,32 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>feature_v19</t>
+          <t>feature_v25_B</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Parental Involvement in Schooling and Academic Monitoring</t>
+          <t>Real-life Self-Satisfaction</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>v19</t>
+          <t>v25_B</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>scale_or_single_item</t>
+          <t>decomposed_subscale</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>v19_1;v19_2;v19_3;v19_4;v19_5;v19_6;v19_7;v19_8;v19_9;v19_10</t>
+          <t>v25_4;v25_5;v25_6</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>-0.0725</t>
+          <t>-0.1134</t>
         </is>
       </c>
     </row>
@@ -2902,32 +2902,32 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>feature_v1_male</t>
+          <t>feature_v25_C</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Gender: Male (vs Female)</t>
+          <t>Online-Offline Discrepancy &amp; Immersion</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>v1_male</t>
+          <t>v25_C</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>categorical_dummy</t>
+          <t>decomposed_subscale</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v25_7;v25_8;v25_9;v25_10;v25_11;v25_12;v25_13;v25_14;v25_15</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>-0.1589</t>
+          <t>0.0733</t>
         </is>
       </c>
     </row>
@@ -2944,17 +2944,17 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>feature_v3</t>
+          <t>feature_v34</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Perceived Social Status (Subjective Social Status)</t>
+          <t>Offline Bullying Victimization</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v34</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
@@ -2964,12 +2964,12 @@
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v34</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>0.0091</t>
+          <t>0.0156</t>
         </is>
       </c>
     </row>
@@ -2986,32 +2986,32 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>feature_v23_A</t>
+          <t>feature_v19</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Selective Positive Sharing</t>
+          <t>Parental Involvement in Schooling and Academic Monitoring</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>v23_A</t>
+          <t>v19</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>decomposed_subscale</t>
+          <t>scale_or_single_item</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>v23_1;v23_2;v23_3</t>
+          <t>v19_1;v19_2;v19_3;v19_4;v19_5;v19_6;v19_7;v19_8;v19_9;v19_10</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>0.0826</t>
+          <t>-0.0597</t>
         </is>
       </c>
     </row>
@@ -3028,32 +3028,32 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>feature_v23_B</t>
+          <t>feature_v1_male</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Digital Image Enhancement</t>
+          <t>Gender: Male (vs Female)</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>v23_B</t>
+          <t>v1_male</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>decomposed_subscale</t>
+          <t>categorical_dummy</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>v23_4;v23_5;v23_6</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>-0.0123</t>
+          <t>-0.1627</t>
         </is>
       </c>
     </row>
@@ -3070,32 +3070,32 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>feature_v23_C</t>
+          <t>feature_v3</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Social Feedback Dependency</t>
+          <t>Perceived Social Status (Subjective Social Status)</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>v23_C</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>decomposed_subscale</t>
+          <t>scale_or_single_item</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>v23_7;v23_8;v23_9</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>-0.0124</t>
+          <t>0.0062</t>
         </is>
       </c>
     </row>
@@ -3112,17 +3112,17 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>feature_v36</t>
+          <t>feature_v9</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Physical/Offline Bullying Perpetration</t>
+          <t>School Belonging and School Identification</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>v36</t>
+          <t>v9</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
@@ -3132,12 +3132,12 @@
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>v36</t>
+          <t>v9_1;v9_2;v9_3</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>0.0545</t>
+          <t>-0.0694</t>
         </is>
       </c>
     </row>
@@ -3154,32 +3154,32 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>feature_v26_A</t>
+          <t>feature_v12</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Online Upward Social Comparison</t>
+          <t>Classmate Support and Trust</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>v26_A</t>
+          <t>v12</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>decomposed_subscale</t>
+          <t>scale_or_single_item</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>v26_1;v26_2;v26_3</t>
+          <t>v12_1;v12_2;v12_3</t>
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>0.0043</t>
+          <t>-0.0352</t>
         </is>
       </c>
     </row>
@@ -3196,32 +3196,32 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>feature_v26_B</t>
+          <t>feature_v8_03-v8_06</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Online Perspective Seeking</t>
+          <t>School Social Adversity and Peer Stress Events</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>v26_B</t>
+          <t>v8_03-v8_06</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>decomposed_subscale</t>
+          <t>direct_feature</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>v26_4;v26_5;v26_6</t>
+          <t>v8_03;v8_04;v8_05;v8_06</t>
         </is>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>0.1436</t>
+          <t>0.1581</t>
         </is>
       </c>
     </row>
@@ -3238,17 +3238,17 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>feature_v54_A</t>
+          <t>feature_v23_A</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Self-Awareness</t>
+          <t>Selective Positive Sharing</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>v54_A</t>
+          <t>v23_A</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
@@ -3258,12 +3258,12 @@
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>v54_1;v54_2;v54_3;v54_18</t>
+          <t>v23_1;v23_2;v23_3</t>
         </is>
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>0.2763</t>
+          <t>0.0796</t>
         </is>
       </c>
     </row>
@@ -3280,17 +3280,17 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>feature_v54_B</t>
+          <t>feature_v23_B</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Self-Management</t>
+          <t>Authentic and Less-Ideal Self-Presentation</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>v54_B</t>
+          <t>v23_B</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
@@ -3300,12 +3300,12 @@
       </c>
       <c r="G56" s="3" t="inlineStr">
         <is>
-          <t>v54_4;v54_5;v54_6</t>
+          <t>v23_4;v23_5;v23_6</t>
         </is>
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>-0.1227</t>
+          <t>-0.0117</t>
         </is>
       </c>
     </row>
@@ -3322,17 +3322,17 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>feature_v54_C</t>
+          <t>feature_v23_C</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Motivation &amp; Goal Setting</t>
+          <t>Covert Social Media Monitoring and Passive Participation</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>v54_C</t>
+          <t>v23_C</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
@@ -3342,12 +3342,12 @@
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>v54_7;v54_8;v54_9</t>
+          <t>v23_7;v23_8;v23_9</t>
         </is>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>0.0908</t>
+          <t>-0.0112</t>
         </is>
       </c>
     </row>
@@ -3364,32 +3364,32 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>feature_v54_D</t>
+          <t>feature_v36</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Social Awareness &amp; Relationship Skills</t>
+          <t>Offline Bullying Perpetration</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>v54_D</t>
+          <t>v36</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>decomposed_subscale</t>
+          <t>scale_or_single_item</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>v54_10;v54_11;v54_13;v54_14;v54_15</t>
+          <t>v36</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>-0.0291</t>
+          <t>0.0433</t>
         </is>
       </c>
     </row>
@@ -3406,17 +3406,17 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>feature_v54_E</t>
+          <t>feature_v26_A</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Help-Seeking</t>
+          <t>Online Upward Social Comparison</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>v54_E</t>
+          <t>v26_A</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
@@ -3426,12 +3426,12 @@
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>v54_12;v54_16</t>
+          <t>v26_1;v26_2;v26_3</t>
         </is>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>-0.1101</t>
+          <t>0.0016</t>
         </is>
       </c>
     </row>
@@ -3448,17 +3448,17 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>feature_v54_F</t>
+          <t>feature_v26_B</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Responsible Decision-Making</t>
+          <t>Online Perspective Seeking</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>v54_F</t>
+          <t>v26_B</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
@@ -3468,12 +3468,12 @@
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>v54_17;v54_19;v54_20</t>
+          <t>v26_4;v26_5;v26_6</t>
         </is>
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>-0.0084</t>
+          <t>0.1451</t>
         </is>
       </c>
     </row>
@@ -3490,32 +3490,284 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
+          <t>feature_v54_A</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>Self-Awareness</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>v54_A</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>decomposed_subscale</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>v54_1;v54_2;v54_3</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>0.2234</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>W2 -&gt; W3</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>w2_predict_w3</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>feature_v54_B</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Self-Management</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>v54_B</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>decomposed_subscale</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>v54_4;v54_5;v54_6</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>-0.1157</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>W2 -&gt; W3</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>w2_predict_w3</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>feature_v54_C</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>Motivation &amp; Goal Setting</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>v54_C</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>decomposed_subscale</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>v54_7;v54_8;v54_9</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>0.0816</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>W2 -&gt; W3</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>w2_predict_w3</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>feature_v54_D</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>Social Awareness &amp; Relationship Skills</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>v54_D</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>decomposed_subscale</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>v54_10;v54_11;v54_13;v54_14;v54_15</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>-0.0114</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>W2 -&gt; W3</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>w2_predict_w3</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>feature_v54_E</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Help-Seeking</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>v54_E</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>decomposed_subscale</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>v54_12;v54_16</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>-0.1168</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>W2 -&gt; W3</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>w2_predict_w3</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>feature_v54_F</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>Responsible Decision-Making</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>v54_F</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>decomposed_subscale</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>v54_17;v54_18;v54_19;v54_20</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>0.0554</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>W2 -&gt; W3</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>w2_predict_w3</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
           <t>feature_v22</t>
         </is>
       </c>
-      <c r="D61" s="3" t="inlineStr">
-        <is>
-          <t>Online Coping and Support Seeking under Distress</t>
-        </is>
-      </c>
-      <c r="E61" s="3" t="inlineStr">
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Online Coping and Emotion Regulation under Distress</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
         <is>
           <t>v22</t>
         </is>
       </c>
-      <c r="F61" s="3" t="inlineStr">
+      <c r="F67" s="3" t="inlineStr">
         <is>
           <t>scale_or_single_item</t>
         </is>
       </c>
-      <c r="G61" s="3" t="inlineStr">
+      <c r="G67" s="3" t="inlineStr">
         <is>
           <t>v22_1;v22_2;v22_3;v22_4;v22_5;v22_6</t>
         </is>
       </c>
-      <c r="H61" s="3" t="inlineStr">
-        <is>
-          <t>0.0330</t>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>0.0229</t>
         </is>
       </c>
     </row>
@@ -3541,7 +3793,7 @@
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
@@ -3640,7 +3892,7 @@
         <v>6603</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
@@ -3654,13 +3906,13 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>v52_health</t>
+          <t>v52_health;v8_03-v8_06</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr"/>
       <c r="K2" s="3" t="inlineStr"/>
       <c r="L2" s="3" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>6603</v>
@@ -3691,7 +3943,7 @@
         <v>6603</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
@@ -3705,13 +3957,13 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>v52_health</t>
+          <t>v52_health;v8_03-v8_06</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr"/>
       <c r="K3" s="3" t="inlineStr"/>
       <c r="L3" s="3" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>6603</v>

</xml_diff>